<commit_message>
chore(examples): align trio outputs and fix textbox schema usage
- Rename every script's output to match its name-aligned trio
  (formulas.sh→formulas.docx, charts.sh→charts.xlsx, etc.) and
  use $(dirname "$0") so outputs always land next to the script
  regardless of caller CWD.
- tables.sh produces a 3-format demo so its xlsx/pptx are renamed to
  tables.{xlsx,pptx} alongside tables.docx.
- 3d-model.sh: fix nonexistent outputs/ subpath.
- textbox.sh: append paragraphs via "//w:body/w:sectPr"+insertbefore
  instead of "//w:body"+append, since w:sectPr must be the last
  child of w:body. Final document now validates clean.
- Add missing numbering-showcase.md stub to complete the trio.
- Refresh README.md to match real script names and current help-command
  syntax (officecli help <fmt> ...).
</commit_message>
<xml_diff>
--- a/examples/excel/charts-demo.xlsx
+++ b/examples/excel/charts-demo.xlsx
@@ -1030,7 +1030,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R5cb1a569784d4612"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rc7972f3bf1d14dbb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1060,7 +1060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rf7272bd1e81a4b66"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R9fda1337d27d4851"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1090,7 +1090,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R55548c4dcacc4a92"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R072548c96c004b93"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1120,7 +1120,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R57224e7b28fa495b"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rab5e11410f4e418a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1150,7 +1150,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R90d0b95ef7dd4a29"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R807d78cec5b14d11"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1180,7 +1180,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R1886a573335f460b"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R743038bfe9cc46bc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1190,7 +1190,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="str">
@@ -1414,6 +1414,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad04320dbbc4197"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978b7432b9214587"/>
 </x:worksheet>
 </file>
</xml_diff>